<commit_message>
scan time excel overview updated
</commit_message>
<xml_diff>
--- a/experiment/docs/scan_time_calculator.xlsx
+++ b/experiment/docs/scan_time_calculator.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yavuz Karaca\PycharmProjects\ArcRuleGenerator\experiment\fMRI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yavuz Karaca\PycharmProjects\arc-fmri\experiment\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6484B51-D801-42F8-8F13-6B9054376D45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{401786EB-4763-42A4-9D2B-2CC37F5211CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10596" yWindow="1200" windowWidth="15912" windowHeight="13644" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14964" yWindow="1752" windowWidth="14868" windowHeight="10920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Scan Time Calculator" sheetId="1" r:id="rId1"/>
@@ -647,7 +647,7 @@
         <v>15</v>
       </c>
       <c r="B7" s="6">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>5</v>
@@ -676,7 +676,7 @@
       </c>
       <c r="B10" s="9">
         <f>(B9*B4)+B7</f>
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -697,7 +697,7 @@
       </c>
       <c r="B13" s="9">
         <f>(B12*B10)+ (B7*2)</f>
-        <v>520</v>
+        <v>485</v>
       </c>
       <c r="D13" t="s">
         <v>16</v>
@@ -709,7 +709,7 @@
       </c>
       <c r="B14" s="17">
         <f>B13/60</f>
-        <v>8.6666666666666661</v>
+        <v>8.0833333333333339</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
@@ -721,7 +721,7 @@
         <v>11</v>
       </c>
       <c r="B16" s="6">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
@@ -730,7 +730,7 @@
       </c>
       <c r="B17" s="16">
         <f>(B16*B13)/60</f>
-        <v>52</v>
+        <v>64.666666666666671</v>
       </c>
     </row>
   </sheetData>

</xml_diff>